<commit_message>
solve conflict and bugs
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA686453-46A7-46E0-98DD-1D2973C5800A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5369CCE2-FA5B-4DAB-9BAA-964595DC84BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -5767,10 +5767,10 @@
         <v>46197</v>
       </c>
       <c r="E265" s="2">
-        <v>0.33333333333333331</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="F265" s="2">
-        <v>0.70833333333333337</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat: cập nhật logic chấm công OT và việt hoá giao diện
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\SWP_GROUP2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FPT\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602B32A4-B075-4FB3-9041-1AD201E27435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA324C77-3F83-4004-AAFB-A34D8F4B418A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1446" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="57">
   <si>
     <t>employeeCode</t>
   </si>
@@ -564,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F271"/>
+  <dimension ref="A1:F211"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -1771,8 +1771,8 @@
       <c r="E60" t="s">
         <v>10</v>
       </c>
-      <c r="F60" t="s">
-        <v>11</v>
+      <c r="F60" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -1797,13 +1797,13 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B62" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C62" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D62" t="s">
         <v>9</v>
@@ -1817,13 +1817,13 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B63" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C63" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
@@ -1837,13 +1837,13 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B64" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C64" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D64" t="s">
         <v>14</v>
@@ -1857,13 +1857,13 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B65" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C65" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D65" t="s">
         <v>15</v>
@@ -1877,13 +1877,13 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B66" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C66" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D66" t="s">
         <v>16</v>
@@ -1897,13 +1897,13 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B67" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C67" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D67" t="s">
         <v>17</v>
@@ -1917,13 +1917,13 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B68" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C68" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D68" t="s">
         <v>19</v>
@@ -1937,13 +1937,13 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B69" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C69" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D69" t="s">
         <v>20</v>
@@ -1957,13 +1957,13 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B70" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C70" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D70" t="s">
         <v>21</v>
@@ -1977,13 +1977,13 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B71" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C71" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D71" t="s">
         <v>22</v>
@@ -1997,13 +1997,13 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B72" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C72" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D72" t="s">
         <v>23</v>
@@ -2017,13 +2017,13 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B73" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C73" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D73" t="s">
         <v>24</v>
@@ -2037,13 +2037,13 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B74" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C74" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D74" t="s">
         <v>25</v>
@@ -2057,13 +2057,13 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B75" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C75" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D75" t="s">
         <v>26</v>
@@ -2077,13 +2077,13 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B76" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C76" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D76" t="s">
         <v>27</v>
@@ -2097,13 +2097,13 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B77" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C77" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D77" t="s">
         <v>28</v>
@@ -2117,13 +2117,13 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B78" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C78" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D78" t="s">
         <v>29</v>
@@ -2137,13 +2137,13 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B79" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C79" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D79" t="s">
         <v>30</v>
@@ -2157,13 +2157,13 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B80" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C80" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D80" t="s">
         <v>31</v>
@@ -2177,13 +2177,13 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B81" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C81" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D81" t="s">
         <v>32</v>
@@ -2197,13 +2197,13 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B82" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C82" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D82" t="s">
         <v>33</v>
@@ -2217,13 +2217,13 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B83" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C83" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D83" t="s">
         <v>34</v>
@@ -2237,13 +2237,13 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B84" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C84" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D84" t="s">
         <v>35</v>
@@ -2257,13 +2257,13 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B85" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C85" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D85" t="s">
         <v>36</v>
@@ -2277,13 +2277,13 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B86" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C86" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D86" t="s">
         <v>37</v>
@@ -2297,13 +2297,13 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B87" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C87" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D87" t="s">
         <v>38</v>
@@ -2317,13 +2317,13 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B88" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C88" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D88" t="s">
         <v>39</v>
@@ -2337,13 +2337,13 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B89" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C89" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D89" t="s">
         <v>40</v>
@@ -2357,13 +2357,13 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B90" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C90" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D90" t="s">
         <v>41</v>
@@ -2377,13 +2377,13 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="B91" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C91" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D91" t="s">
         <v>42</v>
@@ -2397,13 +2397,13 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B92" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C92" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D92" t="s">
         <v>9</v>
@@ -2417,13 +2417,13 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B93" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C93" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D93" t="s">
         <v>12</v>
@@ -2437,13 +2437,13 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B94" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C94" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D94" t="s">
         <v>14</v>
@@ -2457,13 +2457,13 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B95" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C95" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D95" t="s">
         <v>15</v>
@@ -2477,13 +2477,13 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B96" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C96" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D96" t="s">
         <v>16</v>
@@ -2497,13 +2497,13 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B97" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C97" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D97" t="s">
         <v>17</v>
@@ -2517,13 +2517,13 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B98" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C98" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D98" t="s">
         <v>19</v>
@@ -2537,13 +2537,13 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B99" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C99" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D99" t="s">
         <v>20</v>
@@ -2557,13 +2557,13 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B100" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C100" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D100" t="s">
         <v>21</v>
@@ -2577,13 +2577,13 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B101" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C101" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D101" t="s">
         <v>22</v>
@@ -2597,13 +2597,13 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B102" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C102" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D102" t="s">
         <v>23</v>
@@ -2617,13 +2617,13 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B103" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C103" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D103" t="s">
         <v>24</v>
@@ -2637,13 +2637,13 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B104" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C104" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D104" t="s">
         <v>25</v>
@@ -2657,13 +2657,13 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B105" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C105" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D105" t="s">
         <v>26</v>
@@ -2677,13 +2677,13 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B106" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C106" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D106" t="s">
         <v>27</v>
@@ -2697,13 +2697,13 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B107" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C107" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D107" t="s">
         <v>28</v>
@@ -2717,13 +2717,13 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B108" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C108" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D108" t="s">
         <v>29</v>
@@ -2737,13 +2737,13 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B109" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C109" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D109" t="s">
         <v>30</v>
@@ -2757,13 +2757,13 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B110" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C110" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D110" t="s">
         <v>31</v>
@@ -2777,13 +2777,13 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B111" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C111" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D111" t="s">
         <v>32</v>
@@ -2797,13 +2797,13 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B112" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C112" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D112" t="s">
         <v>33</v>
@@ -2817,13 +2817,13 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B113" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C113" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D113" t="s">
         <v>34</v>
@@ -2837,13 +2837,13 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B114" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C114" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D114" t="s">
         <v>35</v>
@@ -2857,13 +2857,13 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B115" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C115" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D115" t="s">
         <v>36</v>
@@ -2877,13 +2877,13 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B116" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C116" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D116" t="s">
         <v>37</v>
@@ -2897,13 +2897,13 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B117" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C117" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D117" t="s">
         <v>38</v>
@@ -2917,13 +2917,13 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B118" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C118" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D118" t="s">
         <v>39</v>
@@ -2937,13 +2937,13 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B119" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C119" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D119" t="s">
         <v>40</v>
@@ -2957,13 +2957,13 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B120" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C120" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D120" t="s">
         <v>41</v>
@@ -2977,13 +2977,13 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B121" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C121" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="D121" t="s">
         <v>42</v>
@@ -2997,10 +2997,10 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B122" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C122" t="s">
         <v>47</v>
@@ -3017,10 +3017,10 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B123" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C123" t="s">
         <v>47</v>
@@ -3037,10 +3037,10 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B124" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C124" t="s">
         <v>47</v>
@@ -3057,10 +3057,10 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B125" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C125" t="s">
         <v>47</v>
@@ -3077,10 +3077,10 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B126" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C126" t="s">
         <v>47</v>
@@ -3097,10 +3097,10 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B127" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C127" t="s">
         <v>47</v>
@@ -3117,10 +3117,10 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B128" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C128" t="s">
         <v>47</v>
@@ -3137,10 +3137,10 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B129" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C129" t="s">
         <v>47</v>
@@ -3157,10 +3157,10 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B130" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C130" t="s">
         <v>47</v>
@@ -3177,10 +3177,10 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B131" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C131" t="s">
         <v>47</v>
@@ -3197,10 +3197,10 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B132" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C132" t="s">
         <v>47</v>
@@ -3217,10 +3217,10 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B133" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C133" t="s">
         <v>47</v>
@@ -3237,10 +3237,10 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B134" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C134" t="s">
         <v>47</v>
@@ -3257,10 +3257,10 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B135" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C135" t="s">
         <v>47</v>
@@ -3277,10 +3277,10 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B136" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C136" t="s">
         <v>47</v>
@@ -3297,10 +3297,10 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B137" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C137" t="s">
         <v>47</v>
@@ -3317,10 +3317,10 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B138" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C138" t="s">
         <v>47</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B139" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C139" t="s">
         <v>47</v>
@@ -3357,10 +3357,10 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B140" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C140" t="s">
         <v>47</v>
@@ -3377,10 +3377,10 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B141" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C141" t="s">
         <v>47</v>
@@ -3397,10 +3397,10 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B142" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C142" t="s">
         <v>47</v>
@@ -3417,10 +3417,10 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B143" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C143" t="s">
         <v>47</v>
@@ -3437,10 +3437,10 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B144" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C144" t="s">
         <v>47</v>
@@ -3457,10 +3457,10 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B145" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C145" t="s">
         <v>47</v>
@@ -3477,10 +3477,10 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B146" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C146" t="s">
         <v>47</v>
@@ -3497,10 +3497,10 @@
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B147" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C147" t="s">
         <v>47</v>
@@ -3517,10 +3517,10 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B148" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C148" t="s">
         <v>47</v>
@@ -3537,10 +3537,10 @@
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B149" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C149" t="s">
         <v>47</v>
@@ -3557,10 +3557,10 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B150" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C150" t="s">
         <v>47</v>
@@ -3577,10 +3577,10 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B151" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C151" t="s">
         <v>47</v>
@@ -3597,2281 +3597,1081 @@
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B152" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C152" t="s">
-        <v>47</v>
-      </c>
-      <c r="D152" t="s">
-        <v>9</v>
-      </c>
-      <c r="E152" t="s">
-        <v>10</v>
-      </c>
-      <c r="F152" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D152" s="1">
+        <v>46174</v>
+      </c>
+      <c r="E152" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F152" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B153" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C153" t="s">
-        <v>47</v>
-      </c>
-      <c r="D153" t="s">
-        <v>12</v>
-      </c>
-      <c r="E153" t="s">
-        <v>13</v>
-      </c>
-      <c r="F153" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D153" s="1">
+        <v>46175</v>
+      </c>
+      <c r="E153" s="2">
+        <v>0.34375</v>
+      </c>
+      <c r="F153" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B154" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C154" t="s">
-        <v>47</v>
-      </c>
-      <c r="D154" t="s">
-        <v>14</v>
-      </c>
-      <c r="E154" t="s">
-        <v>10</v>
-      </c>
-      <c r="F154" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D154" s="1">
+        <v>46176</v>
+      </c>
+      <c r="E154" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F154" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B155" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C155" t="s">
-        <v>47</v>
-      </c>
-      <c r="D155" t="s">
-        <v>15</v>
-      </c>
-      <c r="E155" t="s">
-        <v>10</v>
-      </c>
-      <c r="F155" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D155" s="1">
+        <v>46177</v>
+      </c>
+      <c r="E155" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F155" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B156" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C156" t="s">
-        <v>47</v>
-      </c>
-      <c r="D156" t="s">
-        <v>16</v>
-      </c>
-      <c r="E156" t="s">
-        <v>10</v>
-      </c>
-      <c r="F156" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D156" s="1">
+        <v>46178</v>
+      </c>
+      <c r="E156" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F156" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B157" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C157" t="s">
-        <v>47</v>
-      </c>
-      <c r="D157" t="s">
-        <v>17</v>
-      </c>
-      <c r="E157" t="s">
-        <v>18</v>
-      </c>
-      <c r="F157" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D157" s="1">
+        <v>46179</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B158" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C158" t="s">
-        <v>47</v>
-      </c>
-      <c r="D158" t="s">
-        <v>19</v>
-      </c>
-      <c r="E158" t="s">
-        <v>18</v>
-      </c>
-      <c r="F158" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D158" s="1">
+        <v>46180</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B159" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C159" t="s">
-        <v>47</v>
-      </c>
-      <c r="D159" t="s">
-        <v>20</v>
-      </c>
-      <c r="E159" t="s">
-        <v>18</v>
-      </c>
-      <c r="F159" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D159" s="1">
+        <v>46181</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B160" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C160" t="s">
-        <v>47</v>
-      </c>
-      <c r="D160" t="s">
-        <v>21</v>
-      </c>
-      <c r="E160" t="s">
-        <v>10</v>
-      </c>
-      <c r="F160" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D160" s="1">
+        <v>46182</v>
+      </c>
+      <c r="E160" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F160" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B161" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C161" t="s">
-        <v>47</v>
-      </c>
-      <c r="D161" t="s">
-        <v>22</v>
-      </c>
-      <c r="E161" t="s">
-        <v>10</v>
-      </c>
-      <c r="F161" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D161" s="1">
+        <v>46183</v>
+      </c>
+      <c r="E161" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F161" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B162" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C162" t="s">
-        <v>47</v>
-      </c>
-      <c r="D162" t="s">
-        <v>23</v>
-      </c>
-      <c r="E162" t="s">
-        <v>10</v>
-      </c>
-      <c r="F162" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D162" s="1">
+        <v>46184</v>
+      </c>
+      <c r="E162" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F162" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B163" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C163" t="s">
-        <v>47</v>
-      </c>
-      <c r="D163" t="s">
-        <v>24</v>
-      </c>
-      <c r="E163" t="s">
-        <v>10</v>
-      </c>
-      <c r="F163" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D163" s="1">
+        <v>46185</v>
+      </c>
+      <c r="E163" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F163" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B164" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C164" t="s">
-        <v>47</v>
-      </c>
-      <c r="D164" t="s">
-        <v>25</v>
-      </c>
-      <c r="E164" t="s">
-        <v>18</v>
-      </c>
-      <c r="F164" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D164" s="1">
+        <v>46186</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B165" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C165" t="s">
-        <v>47</v>
-      </c>
-      <c r="D165" t="s">
-        <v>26</v>
-      </c>
-      <c r="E165" t="s">
-        <v>18</v>
-      </c>
-      <c r="F165" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D165" s="1">
+        <v>46187</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B166" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C166" t="s">
-        <v>47</v>
-      </c>
-      <c r="D166" t="s">
-        <v>27</v>
-      </c>
-      <c r="E166" t="s">
-        <v>13</v>
-      </c>
-      <c r="F166" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D166" s="1">
+        <v>46188</v>
+      </c>
+      <c r="E166" s="2">
+        <v>0.34375</v>
+      </c>
+      <c r="F166" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B167" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C167" t="s">
-        <v>47</v>
-      </c>
-      <c r="D167" t="s">
-        <v>28</v>
-      </c>
-      <c r="E167" t="s">
-        <v>10</v>
-      </c>
-      <c r="F167" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D167" s="1">
+        <v>46189</v>
+      </c>
+      <c r="E167" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F167" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B168" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C168" t="s">
-        <v>47</v>
-      </c>
-      <c r="D168" t="s">
-        <v>29</v>
-      </c>
-      <c r="E168" t="s">
-        <v>10</v>
-      </c>
-      <c r="F168" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D168" s="1">
+        <v>46190</v>
+      </c>
+      <c r="E168" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F168" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B169" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C169" t="s">
-        <v>47</v>
-      </c>
-      <c r="D169" t="s">
-        <v>30</v>
-      </c>
-      <c r="E169" t="s">
-        <v>10</v>
-      </c>
-      <c r="F169" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D169" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E169" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F169" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B170" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C170" t="s">
-        <v>47</v>
-      </c>
-      <c r="D170" t="s">
-        <v>31</v>
-      </c>
-      <c r="E170" t="s">
-        <v>10</v>
-      </c>
-      <c r="F170" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D170" s="1">
+        <v>46192</v>
+      </c>
+      <c r="E170" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F170" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B171" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C171" t="s">
-        <v>47</v>
-      </c>
-      <c r="D171" t="s">
-        <v>32</v>
-      </c>
-      <c r="E171" t="s">
-        <v>18</v>
-      </c>
-      <c r="F171" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D171" s="1">
+        <v>46193</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B172" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C172" t="s">
-        <v>47</v>
-      </c>
-      <c r="D172" t="s">
-        <v>33</v>
-      </c>
-      <c r="E172" t="s">
-        <v>18</v>
-      </c>
-      <c r="F172" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D172" s="1">
+        <v>46194</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B173" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C173" t="s">
-        <v>47</v>
-      </c>
-      <c r="D173" t="s">
-        <v>34</v>
-      </c>
-      <c r="E173" t="s">
-        <v>10</v>
-      </c>
-      <c r="F173" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D173" s="1">
+        <v>46195</v>
+      </c>
+      <c r="E173" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F173" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B174" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C174" t="s">
-        <v>47</v>
-      </c>
-      <c r="D174" t="s">
-        <v>35</v>
-      </c>
-      <c r="E174" t="s">
-        <v>10</v>
-      </c>
-      <c r="F174" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D174" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E174" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F174" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B175" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C175" t="s">
-        <v>47</v>
-      </c>
-      <c r="D175" t="s">
-        <v>36</v>
-      </c>
-      <c r="E175" t="s">
-        <v>10</v>
-      </c>
-      <c r="F175" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D175" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E175" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F175" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B176" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C176" t="s">
-        <v>47</v>
-      </c>
-      <c r="D176" t="s">
-        <v>37</v>
-      </c>
-      <c r="E176" t="s">
-        <v>10</v>
-      </c>
-      <c r="F176" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D176" s="1">
+        <v>46198</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B177" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C177" t="s">
-        <v>47</v>
-      </c>
-      <c r="D177" t="s">
-        <v>38</v>
-      </c>
-      <c r="E177" t="s">
-        <v>10</v>
-      </c>
-      <c r="F177" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D177" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E177" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F177" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B178" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C178" t="s">
-        <v>47</v>
-      </c>
-      <c r="D178" t="s">
-        <v>39</v>
-      </c>
-      <c r="E178" t="s">
-        <v>18</v>
-      </c>
-      <c r="F178" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D178" s="1">
+        <v>46200</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B179" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C179" t="s">
-        <v>47</v>
-      </c>
-      <c r="D179" t="s">
-        <v>40</v>
-      </c>
-      <c r="E179" t="s">
-        <v>18</v>
-      </c>
-      <c r="F179" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D179" s="1">
+        <v>46201</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B180" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C180" t="s">
-        <v>47</v>
-      </c>
-      <c r="D180" t="s">
-        <v>41</v>
-      </c>
-      <c r="E180" t="s">
-        <v>10</v>
-      </c>
-      <c r="F180" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D180" s="1">
+        <v>46202</v>
+      </c>
+      <c r="E180" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F180" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B181" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C181" t="s">
-        <v>47</v>
-      </c>
-      <c r="D181" t="s">
-        <v>42</v>
-      </c>
-      <c r="E181" t="s">
-        <v>10</v>
-      </c>
-      <c r="F181" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D181" s="1">
+        <v>46203</v>
+      </c>
+      <c r="E181" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F181" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B182" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C182" t="s">
-        <v>47</v>
-      </c>
-      <c r="D182" t="s">
-        <v>9</v>
-      </c>
-      <c r="E182" t="s">
-        <v>10</v>
-      </c>
-      <c r="F182" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D182" s="1">
+        <v>46174</v>
+      </c>
+      <c r="E182" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F182" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B183" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C183" t="s">
-        <v>47</v>
-      </c>
-      <c r="D183" t="s">
-        <v>12</v>
-      </c>
-      <c r="E183" t="s">
-        <v>13</v>
-      </c>
-      <c r="F183" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D183" s="1">
+        <v>46175</v>
+      </c>
+      <c r="E183" s="2">
+        <v>0.34375</v>
+      </c>
+      <c r="F183" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B184" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C184" t="s">
-        <v>47</v>
-      </c>
-      <c r="D184" t="s">
-        <v>14</v>
-      </c>
-      <c r="E184" t="s">
-        <v>10</v>
-      </c>
-      <c r="F184" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D184" s="1">
+        <v>46176</v>
+      </c>
+      <c r="E184" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F184" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B185" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C185" t="s">
-        <v>47</v>
-      </c>
-      <c r="D185" t="s">
-        <v>15</v>
-      </c>
-      <c r="E185" t="s">
-        <v>10</v>
-      </c>
-      <c r="F185" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D185" s="1">
+        <v>46177</v>
+      </c>
+      <c r="E185" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F185" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B186" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C186" t="s">
-        <v>47</v>
-      </c>
-      <c r="D186" t="s">
-        <v>16</v>
-      </c>
-      <c r="E186" t="s">
-        <v>10</v>
-      </c>
-      <c r="F186" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D186" s="1">
+        <v>46178</v>
+      </c>
+      <c r="E186" s="2"/>
+      <c r="F186" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B187" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C187" t="s">
-        <v>47</v>
-      </c>
-      <c r="D187" t="s">
-        <v>17</v>
-      </c>
-      <c r="E187" t="s">
-        <v>18</v>
-      </c>
-      <c r="F187" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D187" s="1">
+        <v>46179</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B188" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C188" t="s">
-        <v>47</v>
-      </c>
-      <c r="D188" t="s">
-        <v>19</v>
-      </c>
-      <c r="E188" t="s">
-        <v>18</v>
-      </c>
-      <c r="F188" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D188" s="1">
+        <v>46180</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B189" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C189" t="s">
-        <v>47</v>
-      </c>
-      <c r="D189" t="s">
-        <v>20</v>
-      </c>
-      <c r="E189" t="s">
-        <v>18</v>
-      </c>
-      <c r="F189" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D189" s="1">
+        <v>46181</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B190" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C190" t="s">
-        <v>47</v>
-      </c>
-      <c r="D190" t="s">
-        <v>21</v>
-      </c>
-      <c r="E190" t="s">
-        <v>10</v>
-      </c>
-      <c r="F190" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D190" s="1">
+        <v>46182</v>
+      </c>
+      <c r="E190" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F190" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B191" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C191" t="s">
-        <v>47</v>
-      </c>
-      <c r="D191" t="s">
-        <v>22</v>
-      </c>
-      <c r="E191" t="s">
-        <v>10</v>
-      </c>
-      <c r="F191" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D191" s="1">
+        <v>46183</v>
+      </c>
+      <c r="E191" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F191" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B192" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C192" t="s">
-        <v>47</v>
-      </c>
-      <c r="D192" t="s">
-        <v>23</v>
-      </c>
-      <c r="E192" t="s">
-        <v>10</v>
-      </c>
-      <c r="F192" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D192" s="1">
+        <v>46184</v>
+      </c>
+      <c r="E192" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F192" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B193" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C193" t="s">
-        <v>47</v>
-      </c>
-      <c r="D193" t="s">
-        <v>24</v>
-      </c>
-      <c r="E193" t="s">
-        <v>10</v>
-      </c>
-      <c r="F193" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D193" s="1">
+        <v>46185</v>
+      </c>
+      <c r="E193" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F193" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B194" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C194" t="s">
-        <v>47</v>
-      </c>
-      <c r="D194" t="s">
-        <v>25</v>
-      </c>
-      <c r="E194" t="s">
-        <v>18</v>
-      </c>
-      <c r="F194" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D194" s="1">
+        <v>46186</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B195" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C195" t="s">
-        <v>47</v>
-      </c>
-      <c r="D195" t="s">
-        <v>26</v>
-      </c>
-      <c r="E195" t="s">
-        <v>18</v>
-      </c>
-      <c r="F195" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D195" s="1">
+        <v>46187</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B196" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C196" t="s">
-        <v>47</v>
-      </c>
-      <c r="D196" t="s">
-        <v>27</v>
-      </c>
-      <c r="E196" t="s">
-        <v>13</v>
-      </c>
-      <c r="F196" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D196" s="1">
+        <v>46188</v>
+      </c>
+      <c r="E196" s="2">
+        <v>0.34375</v>
+      </c>
+      <c r="F196" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B197" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C197" t="s">
-        <v>47</v>
-      </c>
-      <c r="D197" t="s">
-        <v>28</v>
-      </c>
-      <c r="E197" t="s">
-        <v>10</v>
-      </c>
-      <c r="F197" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D197" s="1">
+        <v>46189</v>
+      </c>
+      <c r="E197" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F197" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B198" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C198" t="s">
-        <v>47</v>
-      </c>
-      <c r="D198" t="s">
-        <v>29</v>
-      </c>
-      <c r="E198" t="s">
-        <v>10</v>
-      </c>
-      <c r="F198" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D198" s="1">
+        <v>46190</v>
+      </c>
+      <c r="E198" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F198" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B199" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C199" t="s">
-        <v>47</v>
-      </c>
-      <c r="D199" t="s">
-        <v>30</v>
-      </c>
-      <c r="E199" t="s">
-        <v>10</v>
-      </c>
-      <c r="F199" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D199" s="1">
+        <v>46191</v>
+      </c>
+      <c r="E199" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F199" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B200" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C200" t="s">
-        <v>47</v>
-      </c>
-      <c r="D200" t="s">
-        <v>31</v>
-      </c>
-      <c r="E200" t="s">
-        <v>10</v>
-      </c>
-      <c r="F200" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D200" s="1">
+        <v>46192</v>
+      </c>
+      <c r="E200" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F200" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B201" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C201" t="s">
-        <v>47</v>
-      </c>
-      <c r="D201" t="s">
-        <v>32</v>
-      </c>
-      <c r="E201" t="s">
-        <v>18</v>
-      </c>
-      <c r="F201" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D201" s="1">
+        <v>46193</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B202" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C202" t="s">
-        <v>47</v>
-      </c>
-      <c r="D202" t="s">
-        <v>33</v>
-      </c>
-      <c r="E202" t="s">
-        <v>18</v>
-      </c>
-      <c r="F202" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D202" s="1">
+        <v>46194</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B203" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C203" t="s">
-        <v>47</v>
-      </c>
-      <c r="D203" t="s">
-        <v>34</v>
-      </c>
-      <c r="E203" t="s">
-        <v>10</v>
-      </c>
-      <c r="F203" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D203" s="1">
+        <v>46195</v>
+      </c>
+      <c r="E203" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F203" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B204" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C204" t="s">
-        <v>47</v>
-      </c>
-      <c r="D204" t="s">
-        <v>35</v>
-      </c>
-      <c r="E204" t="s">
-        <v>10</v>
-      </c>
-      <c r="F204" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D204" s="1">
+        <v>46196</v>
+      </c>
+      <c r="E204" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F204" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B205" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C205" t="s">
-        <v>47</v>
-      </c>
-      <c r="D205" t="s">
-        <v>36</v>
-      </c>
-      <c r="E205" t="s">
-        <v>10</v>
-      </c>
-      <c r="F205" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D205" s="1">
+        <v>46197</v>
+      </c>
+      <c r="E205" s="2">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="F205" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B206" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C206" t="s">
-        <v>47</v>
-      </c>
-      <c r="D206" t="s">
-        <v>37</v>
-      </c>
-      <c r="E206" t="s">
-        <v>10</v>
-      </c>
-      <c r="F206" t="s">
-        <v>11</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="D206" s="1">
+        <v>46198</v>
+      </c>
+      <c r="E206" s="2"/>
+      <c r="F206" s="2"/>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B207" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C207" t="s">
-        <v>47</v>
-      </c>
-      <c r="D207" t="s">
-        <v>38</v>
-      </c>
-      <c r="E207" t="s">
-        <v>10</v>
-      </c>
-      <c r="F207" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D207" s="1">
+        <v>46199</v>
+      </c>
+      <c r="E207" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F207" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B208" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C208" t="s">
-        <v>47</v>
-      </c>
-      <c r="D208" t="s">
-        <v>39</v>
-      </c>
-      <c r="E208" t="s">
-        <v>18</v>
-      </c>
-      <c r="F208" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D208" s="1">
+        <v>46200</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B209" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C209" t="s">
-        <v>47</v>
-      </c>
-      <c r="D209" t="s">
-        <v>40</v>
-      </c>
-      <c r="E209" t="s">
-        <v>18</v>
-      </c>
-      <c r="F209" t="s">
-        <v>18</v>
+        <v>54</v>
+      </c>
+      <c r="D209" s="1">
+        <v>46201</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B210" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C210" t="s">
-        <v>47</v>
-      </c>
-      <c r="D210" t="s">
-        <v>41</v>
-      </c>
-      <c r="E210" t="s">
-        <v>10</v>
-      </c>
-      <c r="F210" t="s">
-        <v>11</v>
+        <v>54</v>
+      </c>
+      <c r="D210" s="1">
+        <v>46202</v>
+      </c>
+      <c r="E210" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F210" s="2">
+        <v>0.70833333333333337</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B211" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C211" t="s">
-        <v>47</v>
-      </c>
-      <c r="D211" t="s">
-        <v>42</v>
-      </c>
-      <c r="E211" t="s">
-        <v>10</v>
-      </c>
-      <c r="F211" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A212" t="s">
-        <v>52</v>
-      </c>
-      <c r="B212" t="s">
-        <v>53</v>
-      </c>
-      <c r="C212" t="s">
-        <v>54</v>
-      </c>
-      <c r="D212" s="1">
-        <v>46174</v>
-      </c>
-      <c r="E212" s="2">
+        <v>54</v>
+      </c>
+      <c r="D211" s="1">
+        <v>46203</v>
+      </c>
+      <c r="E211" s="2">
         <v>0.33333333333333331</v>
       </c>
-      <c r="F212" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A213" t="s">
-        <v>52</v>
-      </c>
-      <c r="B213" t="s">
-        <v>53</v>
-      </c>
-      <c r="C213" t="s">
-        <v>54</v>
-      </c>
-      <c r="D213" s="1">
-        <v>46175</v>
-      </c>
-      <c r="E213" s="2">
-        <v>0.34375</v>
-      </c>
-      <c r="F213" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A214" t="s">
-        <v>52</v>
-      </c>
-      <c r="B214" t="s">
-        <v>53</v>
-      </c>
-      <c r="C214" t="s">
-        <v>54</v>
-      </c>
-      <c r="D214" s="1">
-        <v>46176</v>
-      </c>
-      <c r="E214" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F214" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A215" t="s">
-        <v>52</v>
-      </c>
-      <c r="B215" t="s">
-        <v>53</v>
-      </c>
-      <c r="C215" t="s">
-        <v>54</v>
-      </c>
-      <c r="D215" s="1">
-        <v>46177</v>
-      </c>
-      <c r="E215" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F215" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A216" t="s">
-        <v>52</v>
-      </c>
-      <c r="B216" t="s">
-        <v>53</v>
-      </c>
-      <c r="C216" t="s">
-        <v>54</v>
-      </c>
-      <c r="D216" s="1">
-        <v>46178</v>
-      </c>
-      <c r="E216" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F216" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A217" t="s">
-        <v>52</v>
-      </c>
-      <c r="B217" t="s">
-        <v>53</v>
-      </c>
-      <c r="C217" t="s">
-        <v>54</v>
-      </c>
-      <c r="D217" s="1">
-        <v>46179</v>
-      </c>
-    </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A218" t="s">
-        <v>52</v>
-      </c>
-      <c r="B218" t="s">
-        <v>53</v>
-      </c>
-      <c r="C218" t="s">
-        <v>54</v>
-      </c>
-      <c r="D218" s="1">
-        <v>46180</v>
-      </c>
-    </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A219" t="s">
-        <v>52</v>
-      </c>
-      <c r="B219" t="s">
-        <v>53</v>
-      </c>
-      <c r="C219" t="s">
-        <v>54</v>
-      </c>
-      <c r="D219" s="1">
-        <v>46181</v>
-      </c>
-    </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A220" t="s">
-        <v>52</v>
-      </c>
-      <c r="B220" t="s">
-        <v>53</v>
-      </c>
-      <c r="C220" t="s">
-        <v>54</v>
-      </c>
-      <c r="D220" s="1">
-        <v>46182</v>
-      </c>
-      <c r="E220" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F220" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A221" t="s">
-        <v>52</v>
-      </c>
-      <c r="B221" t="s">
-        <v>53</v>
-      </c>
-      <c r="C221" t="s">
-        <v>54</v>
-      </c>
-      <c r="D221" s="1">
-        <v>46183</v>
-      </c>
-      <c r="E221" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F221" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A222" t="s">
-        <v>52</v>
-      </c>
-      <c r="B222" t="s">
-        <v>53</v>
-      </c>
-      <c r="C222" t="s">
-        <v>54</v>
-      </c>
-      <c r="D222" s="1">
-        <v>46184</v>
-      </c>
-      <c r="E222" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F222" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A223" t="s">
-        <v>52</v>
-      </c>
-      <c r="B223" t="s">
-        <v>53</v>
-      </c>
-      <c r="C223" t="s">
-        <v>54</v>
-      </c>
-      <c r="D223" s="1">
-        <v>46185</v>
-      </c>
-      <c r="E223" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F223" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A224" t="s">
-        <v>52</v>
-      </c>
-      <c r="B224" t="s">
-        <v>53</v>
-      </c>
-      <c r="C224" t="s">
-        <v>54</v>
-      </c>
-      <c r="D224" s="1">
-        <v>46186</v>
-      </c>
-    </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A225" t="s">
-        <v>52</v>
-      </c>
-      <c r="B225" t="s">
-        <v>53</v>
-      </c>
-      <c r="C225" t="s">
-        <v>54</v>
-      </c>
-      <c r="D225" s="1">
-        <v>46187</v>
-      </c>
-    </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A226" t="s">
-        <v>52</v>
-      </c>
-      <c r="B226" t="s">
-        <v>53</v>
-      </c>
-      <c r="C226" t="s">
-        <v>54</v>
-      </c>
-      <c r="D226" s="1">
-        <v>46188</v>
-      </c>
-      <c r="E226" s="2">
-        <v>0.34375</v>
-      </c>
-      <c r="F226" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A227" t="s">
-        <v>52</v>
-      </c>
-      <c r="B227" t="s">
-        <v>53</v>
-      </c>
-      <c r="C227" t="s">
-        <v>54</v>
-      </c>
-      <c r="D227" s="1">
-        <v>46189</v>
-      </c>
-      <c r="E227" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F227" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A228" t="s">
-        <v>52</v>
-      </c>
-      <c r="B228" t="s">
-        <v>53</v>
-      </c>
-      <c r="C228" t="s">
-        <v>54</v>
-      </c>
-      <c r="D228" s="1">
-        <v>46190</v>
-      </c>
-      <c r="E228" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F228" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A229" t="s">
-        <v>52</v>
-      </c>
-      <c r="B229" t="s">
-        <v>53</v>
-      </c>
-      <c r="C229" t="s">
-        <v>54</v>
-      </c>
-      <c r="D229" s="1">
-        <v>46191</v>
-      </c>
-      <c r="E229" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F229" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A230" t="s">
-        <v>52</v>
-      </c>
-      <c r="B230" t="s">
-        <v>53</v>
-      </c>
-      <c r="C230" t="s">
-        <v>54</v>
-      </c>
-      <c r="D230" s="1">
-        <v>46192</v>
-      </c>
-      <c r="E230" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F230" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A231" t="s">
-        <v>52</v>
-      </c>
-      <c r="B231" t="s">
-        <v>53</v>
-      </c>
-      <c r="C231" t="s">
-        <v>54</v>
-      </c>
-      <c r="D231" s="1">
-        <v>46193</v>
-      </c>
-    </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A232" t="s">
-        <v>52</v>
-      </c>
-      <c r="B232" t="s">
-        <v>53</v>
-      </c>
-      <c r="C232" t="s">
-        <v>54</v>
-      </c>
-      <c r="D232" s="1">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A233" t="s">
-        <v>52</v>
-      </c>
-      <c r="B233" t="s">
-        <v>53</v>
-      </c>
-      <c r="C233" t="s">
-        <v>54</v>
-      </c>
-      <c r="D233" s="1">
-        <v>46195</v>
-      </c>
-      <c r="E233" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F233" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A234" t="s">
-        <v>52</v>
-      </c>
-      <c r="B234" t="s">
-        <v>53</v>
-      </c>
-      <c r="C234" t="s">
-        <v>54</v>
-      </c>
-      <c r="D234" s="1">
-        <v>46196</v>
-      </c>
-      <c r="E234" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F234" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A235" t="s">
-        <v>52</v>
-      </c>
-      <c r="B235" t="s">
-        <v>53</v>
-      </c>
-      <c r="C235" t="s">
-        <v>54</v>
-      </c>
-      <c r="D235" s="1">
-        <v>46197</v>
-      </c>
-      <c r="E235" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F235" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A236" t="s">
-        <v>52</v>
-      </c>
-      <c r="B236" t="s">
-        <v>53</v>
-      </c>
-      <c r="C236" t="s">
-        <v>54</v>
-      </c>
-      <c r="D236" s="1">
-        <v>46198</v>
-      </c>
-    </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A237" t="s">
-        <v>52</v>
-      </c>
-      <c r="B237" t="s">
-        <v>53</v>
-      </c>
-      <c r="C237" t="s">
-        <v>54</v>
-      </c>
-      <c r="D237" s="1">
-        <v>46199</v>
-      </c>
-      <c r="E237" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F237" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A238" t="s">
-        <v>52</v>
-      </c>
-      <c r="B238" t="s">
-        <v>53</v>
-      </c>
-      <c r="C238" t="s">
-        <v>54</v>
-      </c>
-      <c r="D238" s="1">
-        <v>46200</v>
-      </c>
-    </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A239" t="s">
-        <v>52</v>
-      </c>
-      <c r="B239" t="s">
-        <v>53</v>
-      </c>
-      <c r="C239" t="s">
-        <v>54</v>
-      </c>
-      <c r="D239" s="1">
-        <v>46201</v>
-      </c>
-    </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A240" t="s">
-        <v>52</v>
-      </c>
-      <c r="B240" t="s">
-        <v>53</v>
-      </c>
-      <c r="C240" t="s">
-        <v>54</v>
-      </c>
-      <c r="D240" s="1">
-        <v>46202</v>
-      </c>
-      <c r="E240" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F240" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A241" t="s">
-        <v>52</v>
-      </c>
-      <c r="B241" t="s">
-        <v>53</v>
-      </c>
-      <c r="C241" t="s">
-        <v>54</v>
-      </c>
-      <c r="D241" s="1">
-        <v>46203</v>
-      </c>
-      <c r="E241" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F241" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A242" t="s">
-        <v>55</v>
-      </c>
-      <c r="B242" t="s">
-        <v>56</v>
-      </c>
-      <c r="C242" t="s">
-        <v>54</v>
-      </c>
-      <c r="D242" s="1">
-        <v>46174</v>
-      </c>
-      <c r="E242" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F242" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A243" t="s">
-        <v>55</v>
-      </c>
-      <c r="B243" t="s">
-        <v>56</v>
-      </c>
-      <c r="C243" t="s">
-        <v>54</v>
-      </c>
-      <c r="D243" s="1">
-        <v>46175</v>
-      </c>
-      <c r="E243" s="2">
-        <v>0.34375</v>
-      </c>
-      <c r="F243" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A244" t="s">
-        <v>55</v>
-      </c>
-      <c r="B244" t="s">
-        <v>56</v>
-      </c>
-      <c r="C244" t="s">
-        <v>54</v>
-      </c>
-      <c r="D244" s="1">
-        <v>46176</v>
-      </c>
-      <c r="E244" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F244" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A245" t="s">
-        <v>55</v>
-      </c>
-      <c r="B245" t="s">
-        <v>56</v>
-      </c>
-      <c r="C245" t="s">
-        <v>54</v>
-      </c>
-      <c r="D245" s="1">
-        <v>46177</v>
-      </c>
-      <c r="E245" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F245" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A246" t="s">
-        <v>55</v>
-      </c>
-      <c r="B246" t="s">
-        <v>56</v>
-      </c>
-      <c r="C246" t="s">
-        <v>54</v>
-      </c>
-      <c r="D246" s="1">
-        <v>46178</v>
-      </c>
-      <c r="E246" s="2"/>
-      <c r="F246" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A247" t="s">
-        <v>55</v>
-      </c>
-      <c r="B247" t="s">
-        <v>56</v>
-      </c>
-      <c r="C247" t="s">
-        <v>54</v>
-      </c>
-      <c r="D247" s="1">
-        <v>46179</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A248" t="s">
-        <v>55</v>
-      </c>
-      <c r="B248" t="s">
-        <v>56</v>
-      </c>
-      <c r="C248" t="s">
-        <v>54</v>
-      </c>
-      <c r="D248" s="1">
-        <v>46180</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A249" t="s">
-        <v>55</v>
-      </c>
-      <c r="B249" t="s">
-        <v>56</v>
-      </c>
-      <c r="C249" t="s">
-        <v>54</v>
-      </c>
-      <c r="D249" s="1">
-        <v>46181</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A250" t="s">
-        <v>55</v>
-      </c>
-      <c r="B250" t="s">
-        <v>56</v>
-      </c>
-      <c r="C250" t="s">
-        <v>54</v>
-      </c>
-      <c r="D250" s="1">
-        <v>46182</v>
-      </c>
-      <c r="E250" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F250" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A251" t="s">
-        <v>55</v>
-      </c>
-      <c r="B251" t="s">
-        <v>56</v>
-      </c>
-      <c r="C251" t="s">
-        <v>54</v>
-      </c>
-      <c r="D251" s="1">
-        <v>46183</v>
-      </c>
-      <c r="E251" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F251" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A252" t="s">
-        <v>55</v>
-      </c>
-      <c r="B252" t="s">
-        <v>56</v>
-      </c>
-      <c r="C252" t="s">
-        <v>54</v>
-      </c>
-      <c r="D252" s="1">
-        <v>46184</v>
-      </c>
-      <c r="E252" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F252" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A253" t="s">
-        <v>55</v>
-      </c>
-      <c r="B253" t="s">
-        <v>56</v>
-      </c>
-      <c r="C253" t="s">
-        <v>54</v>
-      </c>
-      <c r="D253" s="1">
-        <v>46185</v>
-      </c>
-      <c r="E253" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F253" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A254" t="s">
-        <v>55</v>
-      </c>
-      <c r="B254" t="s">
-        <v>56</v>
-      </c>
-      <c r="C254" t="s">
-        <v>54</v>
-      </c>
-      <c r="D254" s="1">
-        <v>46186</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A255" t="s">
-        <v>55</v>
-      </c>
-      <c r="B255" t="s">
-        <v>56</v>
-      </c>
-      <c r="C255" t="s">
-        <v>54</v>
-      </c>
-      <c r="D255" s="1">
-        <v>46187</v>
-      </c>
-    </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A256" t="s">
-        <v>55</v>
-      </c>
-      <c r="B256" t="s">
-        <v>56</v>
-      </c>
-      <c r="C256" t="s">
-        <v>54</v>
-      </c>
-      <c r="D256" s="1">
-        <v>46188</v>
-      </c>
-      <c r="E256" s="2">
-        <v>0.34375</v>
-      </c>
-      <c r="F256" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A257" t="s">
-        <v>55</v>
-      </c>
-      <c r="B257" t="s">
-        <v>56</v>
-      </c>
-      <c r="C257" t="s">
-        <v>54</v>
-      </c>
-      <c r="D257" s="1">
-        <v>46189</v>
-      </c>
-      <c r="E257" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F257" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A258" t="s">
-        <v>55</v>
-      </c>
-      <c r="B258" t="s">
-        <v>56</v>
-      </c>
-      <c r="C258" t="s">
-        <v>54</v>
-      </c>
-      <c r="D258" s="1">
-        <v>46190</v>
-      </c>
-      <c r="E258" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F258" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A259" t="s">
-        <v>55</v>
-      </c>
-      <c r="B259" t="s">
-        <v>56</v>
-      </c>
-      <c r="C259" t="s">
-        <v>54</v>
-      </c>
-      <c r="D259" s="1">
-        <v>46191</v>
-      </c>
-      <c r="E259" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F259" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A260" t="s">
-        <v>55</v>
-      </c>
-      <c r="B260" t="s">
-        <v>56</v>
-      </c>
-      <c r="C260" t="s">
-        <v>54</v>
-      </c>
-      <c r="D260" s="1">
-        <v>46192</v>
-      </c>
-      <c r="E260" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F260" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A261" t="s">
-        <v>55</v>
-      </c>
-      <c r="B261" t="s">
-        <v>56</v>
-      </c>
-      <c r="C261" t="s">
-        <v>54</v>
-      </c>
-      <c r="D261" s="1">
-        <v>46193</v>
-      </c>
-    </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A262" t="s">
-        <v>55</v>
-      </c>
-      <c r="B262" t="s">
-        <v>56</v>
-      </c>
-      <c r="C262" t="s">
-        <v>54</v>
-      </c>
-      <c r="D262" s="1">
-        <v>46194</v>
-      </c>
-    </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A263" t="s">
-        <v>55</v>
-      </c>
-      <c r="B263" t="s">
-        <v>56</v>
-      </c>
-      <c r="C263" t="s">
-        <v>54</v>
-      </c>
-      <c r="D263" s="1">
-        <v>46195</v>
-      </c>
-      <c r="E263" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F263" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A264" t="s">
-        <v>55</v>
-      </c>
-      <c r="B264" t="s">
-        <v>56</v>
-      </c>
-      <c r="C264" t="s">
-        <v>54</v>
-      </c>
-      <c r="D264" s="1">
-        <v>46196</v>
-      </c>
-      <c r="E264" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F264" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A265" t="s">
-        <v>55</v>
-      </c>
-      <c r="B265" t="s">
-        <v>56</v>
-      </c>
-      <c r="C265" t="s">
-        <v>54</v>
-      </c>
-      <c r="D265" s="1">
-        <v>46197</v>
-      </c>
-      <c r="E265" s="2">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="F265" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-    </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A266" t="s">
-        <v>55</v>
-      </c>
-      <c r="B266" t="s">
-        <v>56</v>
-      </c>
-      <c r="C266" t="s">
-        <v>54</v>
-      </c>
-      <c r="D266" s="1">
-        <v>46198</v>
-      </c>
-      <c r="E266" s="2"/>
-      <c r="F266" s="2"/>
-    </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A267" t="s">
-        <v>55</v>
-      </c>
-      <c r="B267" t="s">
-        <v>56</v>
-      </c>
-      <c r="C267" t="s">
-        <v>54</v>
-      </c>
-      <c r="D267" s="1">
-        <v>46199</v>
-      </c>
-      <c r="E267" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F267" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A268" t="s">
-        <v>55</v>
-      </c>
-      <c r="B268" t="s">
-        <v>56</v>
-      </c>
-      <c r="C268" t="s">
-        <v>54</v>
-      </c>
-      <c r="D268" s="1">
-        <v>46200</v>
-      </c>
-    </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A269" t="s">
-        <v>55</v>
-      </c>
-      <c r="B269" t="s">
-        <v>56</v>
-      </c>
-      <c r="C269" t="s">
-        <v>54</v>
-      </c>
-      <c r="D269" s="1">
-        <v>46201</v>
-      </c>
-    </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A270" t="s">
-        <v>55</v>
-      </c>
-      <c r="B270" t="s">
-        <v>56</v>
-      </c>
-      <c r="C270" t="s">
-        <v>54</v>
-      </c>
-      <c r="D270" s="1">
-        <v>46202</v>
-      </c>
-      <c r="E270" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F270" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-    </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A271" t="s">
-        <v>55</v>
-      </c>
-      <c r="B271" t="s">
-        <v>56</v>
-      </c>
-      <c r="C271" t="s">
-        <v>54</v>
-      </c>
-      <c r="D271" s="1">
-        <v>46203</v>
-      </c>
-      <c r="E271" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F271" s="2">
+      <c r="F211" s="2">
         <v>0.70833333333333337</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix OT form approver display and validate check-in/out boundaries
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FPT\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383C45E2-8972-4045-90C6-6919EC9B1216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9647F889-5398-4DF2-93E6-D12D41252D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="57">
   <si>
     <t>employeeCode</t>
   </si>
@@ -1377,8 +1377,8 @@
       <c r="E40" t="s">
         <v>10</v>
       </c>
-      <c r="F40" t="s">
-        <v>11</v>
+      <c r="F40" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Fix OT bug: Exact 19:00 checkout now properly revives OT; Removed redundant timeout check for calendar display.
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FPT\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9647F889-5398-4DF2-93E6-D12D41252D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09AC7BE9-AB7C-4F52-9107-13DC1E9E1570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="57">
   <si>
     <t>employeeCode</t>
   </si>
@@ -2837,8 +2837,8 @@
       <c r="E113" t="s">
         <v>10</v>
       </c>
-      <c r="F113" t="s">
-        <v>11</v>
+      <c r="F113" s="2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
@@ -2857,8 +2857,8 @@
       <c r="E114" t="s">
         <v>10</v>
       </c>
-      <c r="F114" t="s">
-        <v>11</v>
+      <c r="F114" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Block duplicate OT assignment for same employee on same date
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FPT\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9647F889-5398-4DF2-93E6-D12D41252D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F73DB68-CD0A-4ED9-8DBD-978822988897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="57">
   <si>
     <t>employeeCode</t>
   </si>
@@ -2837,8 +2837,8 @@
       <c r="E113" t="s">
         <v>10</v>
       </c>
-      <c r="F113" t="s">
-        <v>11</v>
+      <c r="F113" s="2">
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Save stashed work to branch VuPham2
</commit_message>
<xml_diff>
--- a/attendance_demo_FI_2026_06_full.xlsx
+++ b/attendance_demo_FI_2026_06_full.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\SWP_GROUP2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Default\Documents\SWP_GROUP2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB629AB-E401-4E59-8649-F83A74132EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65AC295-F21B-4E1F-B009-7F2816D92D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="12288" windowHeight="8988" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -4633,6 +4633,10 @@
       <c r="D209" s="1">
         <v>46201</v>
       </c>
+      <c r="E209" s="2"/>
+      <c r="F209" s="2">
+        <v>0.70833333333333337</v>
+      </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
@@ -4673,5 +4677,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>